<commit_message>
Record the matched-slice FreeView comparison and the surface QC references used for visual review.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/analysis/QC_checklist.xlsx
+++ b/analysis/QC_checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="90">
   <si>
     <t xml:space="preserve">Subject</t>
   </si>
@@ -217,7 +217,10 @@
     <t xml:space="preserve">mrart_sub-009673_acq-headmotion2_T1w</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass  (great contrast w/still)</t>
+    <t xml:space="preserve">Fail: caudate, hippocampus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good cortical contrast w still</t>
   </si>
   <si>
     <t xml:space="preserve">mrart_sub-010769_acq-headmotion1_T1w</t>
@@ -248,6 +251,9 @@
   </si>
   <si>
     <t xml:space="preserve">mrart_sub-067018_acq-headmotion1_T1w</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">mrart_sub-067018_acq-headmotion2_T1w</t>
@@ -364,7 +370,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -375,6 +381,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -2295,6 +2305,9 @@
       <c r="A22" s="1" t="s">
         <v>47</v>
       </c>
+      <c r="B22" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="O22" s="1" t="n">
         <v>2.85</v>
       </c>
@@ -3631,6 +3644,9 @@
       <c r="B39" s="1" t="s">
         <v>65</v>
       </c>
+      <c r="C39" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="O39" s="1" t="n">
         <v>2.484</v>
       </c>
@@ -3706,7 +3722,7 @@
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="O40" s="1" t="n">
         <v>2.645</v>
@@ -3783,10 +3799,10 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O41" s="1" t="n">
         <v>2.603</v>
@@ -3863,7 +3879,7 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O42" s="1" t="n">
         <v>2.864</v>
@@ -3940,7 +3956,7 @@
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>27</v>
@@ -4020,7 +4036,7 @@
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O44" s="1" t="n">
         <v>2.635</v>
@@ -4097,7 +4113,7 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>27</v>
@@ -4176,8 +4192,8 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
-        <v>73</v>
+      <c r="A46" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="O46" s="1" t="n">
         <v>2.522</v>
@@ -4254,7 +4270,7 @@
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>27</v>
@@ -4334,7 +4350,10 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>77</v>
       </c>
       <c r="O48" s="1" t="n">
         <v>2.852</v>
@@ -4411,7 +4430,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>27</v>
@@ -4491,7 +4510,7 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O50" s="1" t="n">
         <v>2.968</v>
@@ -4568,7 +4587,7 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>27</v>
@@ -4648,7 +4667,7 @@
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>27</v>
@@ -4728,7 +4747,7 @@
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O53" s="1" t="n">
         <v>2.796</v>
@@ -4805,7 +4824,7 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>27</v>
@@ -4885,7 +4904,7 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O55" s="1" t="n">
         <v>2.882</v>
@@ -4962,7 +4981,7 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>27</v>
@@ -5042,7 +5061,7 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O57" s="1" t="n">
         <v>2.935</v>
@@ -5119,7 +5138,7 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>27</v>
@@ -5199,7 +5218,7 @@
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O59" s="1" t="n">
         <v>3.014</v>
@@ -5276,7 +5295,7 @@
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>27</v>

</xml_diff>